<commit_message>
PH-3 A6b: LAUNCH year-plan workbook — 10-hour rule corrected
10 cells, values only, no formulas, no structural change. The workbook asserted a
10-hour plan-use requirement on ComSk1; spec v1.2 places that gate on the other five
PEQ skills (Decision making, Learning, Team working, Thinking, Wellbeing) and gives
Communication activity-time minimums instead.

PEQ Evidence Map E9, A10, B10, E10, A13, A14 · Key Dates & Compliance B7, B21
  (the eight cells proposed in _passph3/JOB_A_REPORT.md)
Autumn Overview D10, D12
  (the same false claim in the PEQ column, MISSED by the JOB_A_REPORT list — the cell
   text never names Communication, so the original proximity scan skipped them)

Verified after: 10-hour-on-Communication assertions 0 (every remaining mention carries
its own in-cell correction); pupil names 0; non-target cell drift NONE; merges,
dimensions and sheet order unchanged.
</commit_message>
<xml_diff>
--- a/Planning/LAUNCH/LAUNCH_Autumn_Year_Plan_ASDAN.xlsx
+++ b/Planning/LAUNCH/LAUNCH_Autumn_Year_Plan_ASDAN.xlsx
@@ -133,7 +133,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -155,11 +155,44 @@
         <color rgb="00C9C9D4"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9C9D4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9C9D4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9C9D4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9C9D4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9C9D4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9C9D4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -230,6 +263,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -627,6 +661,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -795,7 +830,7 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Deliver the activity &amp; gather evidence — PLAN LIVE, 10-hr clock; min 3-min talk OR 250-word text</t>
+          <t>Deliver the activity &amp; gather evidence — PLAN LIVE; ONE activity: min 3-min talk OR 8-min discussion OR 250-word text (no 10-hour rule on Communication)</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -855,7 +890,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Consolidation &amp; gap-fill — 10-hr tally continues  [pattern from BUILD; not in the LAUNCH SoW]</t>
+          <t>Consolidation &amp; gap-fill — plan-use evidence continues across the weeks; no 10-hour tally applies to ComSk1  [pattern from BUILD; not in the LAUNCH SoW]</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -973,6 +1008,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1131,19 +1167,19 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Delivery meeting the ComSk1 minimum — a talk of ≥3 minutes OR a written text of ≥250 words; dated &amp; witnessed. PLAN LIVE — 10-hr clock starts (fixed)</t>
+          <t>Delivery meeting the ComSk1 minimum — ONE activity: a talk of ≥3 minutes OR a discussion of ≥8 minutes OR a written text of ≥250 words; four audience questions prepared in the plan; any group activity needs ≥3 members; dated &amp; witnessed. PLAN LIVE (fixed date)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Use over ≥10 hours</t>
+          <t>Use the plan across the weeks</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Plan used over a minimum of 10 hours</t>
+          <t>Plan used across the weeks — no 10-hour requirement on Communication</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1158,7 +1194,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>10-hour tally logged ACROSS THE WHOLE TIMETABLE by every adult — not the ASDAN slot alone</t>
+          <t>Dated evidence that the plan ran over time, not one lesson. No 10-hour tally is required for ComSk1: the 10-hour plan-use window sits on the other five PEQ skills (Decision making, Learning, Team working, Thinking and Wellbeing), not on Communication.</t>
         </is>
       </c>
     </row>
@@ -1189,20 +1225,22 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>THE 10-HOUR RULE IS THE DESIGN CONSTRAINT</t>
+          <t>COMMUNICATION HAS NO 10-HOUR RULE — THE ACTIVITY MINIMUMS ARE THE CONSTRAINT</t>
         </is>
       </c>
     </row>
     <row r="14" ht="76" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>ComSk1 requires the plan to be USED over a minimum of 10 hours. Those hours accrue across the WHOLE timetable, not the ASDAN slot alone. The plan goes live on a fixed week (w/c 28 Sep) so 10 hours can accrue before the signed review, which completes before the final Aut 1 teaching week (w/c 19 Oct). Brief every adult on the tally before the plan goes live. Note: the deployed lessons state the 3-min / 250-word minimum; a minimum team size is not specified in the built lessons — confirm at the spec check.</t>
-        </is>
-      </c>
-    </row>
+          <t>CORRECTED 2026-08-18 (PH-3, against spec v1.2 Oct 2025). ComSk1 does NOT carry a 10-hour plan-use requirement. That gate — "the plan must be used over a minimum period of 10 hours" — sits on the other five PEQ skills (Decision making, Learning, Team working, Thinking and Wellbeing); Communication carries activity-time minimums instead. What ComSk1 actually requires: ONE activity — a presentation of ≥3 minutes OR a discussion of ≥8 minutes OR a written text of ≥250 words; at least 4 audience questions prepared in the plan, with responses; any group activity needs ≥3 members; and the plan used across the weeks (evidenced over time, not in one lesson). The plan still goes live on a fixed week (w/c 28 Sep) so the across-weeks evidence accrues before the signed review, which completes before the final Aut 1 teaching week (w/c 19 Oct). The earlier note that team size was unspecified is now settled: ≥3 members.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
@@ -1251,6 +1289,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -1269,6 +1308,7 @@
           <t>1 Sep – 18 Dec 2026. FIFTEEN weeks: Aut 1 = 8 weeks, Aut 2 = 7 weeks. LAUNCH content in this plan is Autumn 1.</t>
         </is>
       </c>
+      <c r="C4" s="24" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="20" t="inlineStr">
@@ -1281,6 +1321,7 @@
           <t>Baseline — w/c 1 &amp; 7 Sep. Boxall / GL / BKSB and subject baselines. NO ASDAN assessment.</t>
         </is>
       </c>
+      <c r="C5" s="24" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="20" t="inlineStr">
@@ -1293,6 +1334,7 @@
           <t>ComSk1 teaching underway — w/c 14 Sep.</t>
         </is>
       </c>
+      <c r="C6" s="24" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
@@ -1302,9 +1344,10 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>w/c 28 Sep — PLAN LIVE. 10-hour clock starts. This date is fixed.</t>
-        </is>
-      </c>
+          <t>w/c 28 Sep — PLAN LIVE. This date is fixed. No 10-hour clock: the 10-hour plan-use window does not apply to Communication.</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="20" t="inlineStr">
@@ -1317,6 +1360,7 @@
           <t>w/c 12 Oct — consolidation &amp; gap-fill (pattern from BUILD; not separately in the LAUNCH SoW).</t>
         </is>
       </c>
+      <c r="C8" s="24" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="20" t="inlineStr">
@@ -1329,6 +1373,7 @@
           <t>w/c 19 Oct — LAST WEEK OF AUT 1. Audit: ComSk1 evidence complete &amp; signed.</t>
         </is>
       </c>
+      <c r="C9" s="24" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
@@ -1341,7 +1386,9 @@
           <t>26–30 Oct.</t>
         </is>
       </c>
-    </row>
+      <c r="C10" s="24" t="n"/>
+    </row>
+    <row r="11"/>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
         <is>
@@ -1360,6 +1407,7 @@
           <t>GCSE Biology (Pearson 1BI0, Foundation) or Combined Science (Pearson 1SC0, Foundation); the IGCSE suite as an optional stretch for eligible students.</t>
         </is>
       </c>
+      <c r="C13" s="24" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
@@ -1372,6 +1420,7 @@
           <t>AQA English Language 8700; optional AQA English Literature 8702 and AQA Entry Level Certificate 8145.</t>
         </is>
       </c>
+      <c r="C14" s="24" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
@@ -1384,6 +1433,7 @@
           <t>Trinity Arts Award Silver (Unit 1 + Unit 2).</t>
         </is>
       </c>
+      <c r="C15" s="24" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
@@ -1396,7 +1446,9 @@
           <t>Personal Effectiveness — Entry 3 to Level 1 only in 2026/27 (ComSk1 this term). Other strands bank ASDAN short courses + AQA Unit Award Scheme.</t>
         </is>
       </c>
-    </row>
+      <c r="C16" s="24" t="n"/>
+    </row>
+    <row r="17"/>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
@@ -1415,6 +1467,7 @@
           <t>REGISTER THE COHORT WITH ASDAN before any assessment takes place. No evidence counts until registration is complete. (Cheryl's decision — still open.)</t>
         </is>
       </c>
+      <c r="C19" s="24" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="21" t="inlineStr">
@@ -1427,6 +1480,7 @@
           <t>BOOK FIRST-YEAR EQA SAMPLING. Required in year one even with no completers.</t>
         </is>
       </c>
+      <c r="C20" s="24" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="21" t="inlineStr">
@@ -1436,9 +1490,10 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Brief every adult on the 10-hour tally before the plan goes live.</t>
-        </is>
-      </c>
+          <t>Brief every adult that the plan is live and evidence is gathered across the weeks. No 10-hour tally is required for ComSk1 — that window sits on the other five PEQ skills.</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="21" t="inlineStr">
@@ -1451,6 +1506,7 @@
           <t>Assessment records signed by BOTH assessor AND learner.</t>
         </is>
       </c>
+      <c r="C22" s="24" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="21" t="inlineStr">
@@ -1463,7 +1519,9 @@
           <t>Book the Trinity Arts Award adviser training (Discover &amp; Explore / Silver).</t>
         </is>
       </c>
-    </row>
+      <c r="C23" s="24" t="n"/>
+    </row>
+    <row r="24"/>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="13" t="inlineStr">
         <is>
@@ -1531,6 +1589,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>

</xml_diff>